<commit_message>
Update tissue type to include egg and heart in excel file
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v17.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v17.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{515548F7-397A-3F4D-8340-9C43B7EE9B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEF876F-4FCA-354B-B8EB-E81D3890F2CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
@@ -1357,13 +1357,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1387,6 +1380,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1739,20 +1739,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="43" t="s">
         <v>220</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
     </row>
     <row r="2" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="43" t="s">
         <v>200</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
@@ -2768,27 +2768,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="44" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
       <c r="D1" s="10" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="37"/>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="11" t="s">
         <v>214</v>
       </c>
@@ -2834,27 +2834,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="44" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
       <c r="D1" s="10" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="37"/>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
       <c r="D3" s="11" t="s">
         <v>25</v>
       </c>
@@ -43846,27 +43846,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="44" t="s">
         <v>197</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
       <c r="D1" s="5" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
       <c r="D2" s="6"/>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A3" s="37"/>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
       <c r="D3" s="6" t="s">
         <v>25</v>
       </c>
@@ -43889,163 +43889,163 @@
       </c>
     </row>
     <row r="5" spans="1:53" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="36" t="s">
         <v>81</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="C5" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="38" t="s">
         <v>207</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="G5" s="40" t="s">
+      <c r="G5" s="37" t="s">
         <v>140</v>
       </c>
-      <c r="H5" s="42" t="s">
+      <c r="H5" s="39" t="s">
         <v>203</v>
       </c>
-      <c r="I5" s="42" t="s">
+      <c r="I5" s="39" t="s">
         <v>201</v>
       </c>
-      <c r="J5" s="40" t="s">
+      <c r="J5" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="40" t="s">
+      <c r="K5" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="L5" s="40" t="s">
+      <c r="L5" s="37" t="s">
         <v>204</v>
       </c>
-      <c r="M5" s="40" t="s">
+      <c r="M5" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="N5" s="42" t="s">
+      <c r="N5" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="O5" s="40" t="s">
+      <c r="O5" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="P5" s="40" t="s">
+      <c r="P5" s="37" t="s">
         <v>208</v>
       </c>
-      <c r="Q5" s="40" t="s">
+      <c r="Q5" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="R5" s="40" t="s">
+      <c r="R5" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="S5" s="40" t="s">
+      <c r="S5" s="37" t="s">
         <v>209</v>
       </c>
-      <c r="T5" s="43" t="s">
+      <c r="T5" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="U5" s="43" t="s">
+      <c r="U5" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="V5" s="42" t="s">
+      <c r="V5" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="W5" s="44" t="s">
+      <c r="W5" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="X5" s="43" t="s">
+      <c r="X5" s="40" t="s">
         <v>126</v>
       </c>
-      <c r="Y5" s="42" t="s">
+      <c r="Y5" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="Z5" s="40" t="s">
+      <c r="Z5" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="AA5" s="40" t="s">
+      <c r="AA5" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="AB5" s="40" t="s">
+      <c r="AB5" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="AC5" s="45" t="s">
+      <c r="AC5" s="42" t="s">
         <v>205</v>
       </c>
-      <c r="AD5" s="45" t="s">
+      <c r="AD5" s="42" t="s">
         <v>206</v>
       </c>
-      <c r="AE5" s="45" t="s">
+      <c r="AE5" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="AF5" s="45" t="s">
+      <c r="AF5" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="AG5" s="40" t="s">
+      <c r="AG5" s="37" t="s">
         <v>143</v>
       </c>
-      <c r="AH5" s="40" t="s">
+      <c r="AH5" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="AI5" s="40" t="s">
+      <c r="AI5" s="37" t="s">
         <v>147</v>
       </c>
-      <c r="AJ5" s="40" t="s">
+      <c r="AJ5" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="AK5" s="43" t="s">
+      <c r="AK5" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="AL5" s="43" t="s">
+      <c r="AL5" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="AM5" s="43" t="s">
+      <c r="AM5" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="AN5" s="43" t="s">
+      <c r="AN5" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="AO5" s="40" t="s">
+      <c r="AO5" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AP5" s="40" t="s">
+      <c r="AP5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="AQ5" s="40" t="s">
+      <c r="AQ5" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="AR5" s="40" t="s">
+      <c r="AR5" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="AS5" s="40" t="s">
+      <c r="AS5" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="AT5" s="40" t="s">
+      <c r="AT5" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="AU5" s="40" t="s">
+      <c r="AU5" s="37" t="s">
         <v>228</v>
       </c>
-      <c r="AV5" s="40" t="s">
+      <c r="AV5" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="AW5" s="40" t="s">
+      <c r="AW5" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="AX5" s="40" t="s">
+      <c r="AX5" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="AY5" s="40" t="s">
+      <c r="AY5" s="37" t="s">
         <v>233</v>
       </c>
-      <c r="AZ5" s="40" t="s">
+      <c r="AZ5" s="37" t="s">
         <v>236</v>
       </c>
-      <c r="BA5" s="40" t="s">
+      <c r="BA5" s="37" t="s">
         <v>154</v>
       </c>
     </row>
@@ -44090,7 +44090,7 @@
       <formula1>"fry, larva, juvenile, adult "</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V6:V10000" xr:uid="{783A5061-181E-6647-B48C-F16794E29794}">
-      <formula1>"belly flap, blood, carcass, cleithra, eye lens, fin, gonad, liver, muscle, otolith, scale, spine, stomach, viscera, whole body, whole body (gonads removed), whole body (stomach removed)"</formula1>
+      <formula1>"belly flap, blood, carcass, cleithra, eye lens, egg, fin, gonad, heart, liver, muscle, otolith, scale, spine, stomach, viscera, whole body, whole body (gonads removed), whole body (stomach removed)"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU6:AU10000" xr:uid="{0DD4FFBC-3D6E-914E-8511-DDD8F03F7232}">
       <formula1>"bulk, lipid free"</formula1>

</xml_diff>